<commit_message>
FAQs: two-column layout matching wknd.site
The FAQ page rendered everything stacked with a full-width (1200px) image.
The source uses a two-column layout: main content (heading, image, intro,
accordion) on the left and the "Need more help?" contact in a narrow 291px
column on the right.

- Tag the FAQ section with Style=faqs in the import script
- Add a .section.faqs grid (1fr / 291px) so the contact sits beside the
  content and the image is constrained to the left column

Co-Authored-By: Claude Opus 4.8 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/tools/importer/reports/import-wknd-faqs.report.xlsx
+++ b/tools/importer/reports/import-wknd-faqs.report.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="390" uniqueCount="205">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="620" uniqueCount="274">
   <si>
     <t>_reportFile</t>
   </si>
@@ -163,7 +163,7 @@
     <t>wknd-footer</t>
   </si>
   <si>
-    <t>2026-08-12T10:41:01.214Z</t>
+    <t>2026-08-12T11:10:55.259Z</t>
   </si>
   <si>
     <t>Footer</t>
@@ -208,7 +208,7 @@
     <t>wknd-nav</t>
   </si>
   <si>
-    <t>2026-08-10T10:18:20.500Z</t>
+    <t>2026-08-12T11:10:49.807Z</t>
   </si>
   <si>
     <t>Nav</t>
@@ -592,13 +592,22 @@
     <t>2026-08-12T11:10:28.532Z</t>
   </si>
   <si>
+    <t>us/en/adventures.report.json</t>
+  </si>
+  <si>
+    <t>us/en/adventures</t>
+  </si>
+  <si>
+    <t>2026-08-12T11:10:44.946Z</t>
+  </si>
+  <si>
     <t>us/en/faqs.report.json</t>
   </si>
   <si>
     <t>us/en/faqs</t>
   </si>
   <si>
-    <t>2026-08-12T11:10:39.124Z</t>
+    <t>2026-08-12T11:51:45.004Z</t>
   </si>
   <si>
     <t>us/en/magazine.report.json</t>
@@ -608,6 +617,150 @@
   </si>
   <si>
     <t>2026-08-12T11:10:33.825Z</t>
+  </si>
+  <si>
+    <t>us/en/search.report.json</t>
+  </si>
+  <si>
+    <t>us/en/search</t>
+  </si>
+  <si>
+    <t>2026-08-12T11:11:00.753Z</t>
+  </si>
+  <si>
+    <t>us/en/adventures/bali-surf-camp.report.json</t>
+  </si>
+  <si>
+    <t>us/en/adventures/bali-surf-camp</t>
+  </si>
+  <si>
+    <t>2026-08-12T11:13:39.792Z</t>
+  </si>
+  <si>
+    <t>us/en/adventures/beervana-portland.report.json</t>
+  </si>
+  <si>
+    <t>us/en/adventures/beervana-portland</t>
+  </si>
+  <si>
+    <t>2026-08-12T11:13:44.785Z</t>
+  </si>
+  <si>
+    <t>us/en/adventures/climbing-new-zealand.report.json</t>
+  </si>
+  <si>
+    <t>us/en/adventures/climbing-new-zealand</t>
+  </si>
+  <si>
+    <t>2026-08-12T11:13:50.857Z</t>
+  </si>
+  <si>
+    <t>us/en/adventures/colorado-rock-climbing.report.json</t>
+  </si>
+  <si>
+    <t>us/en/adventures/colorado-rock-climbing</t>
+  </si>
+  <si>
+    <t>2026-08-12T11:13:56.233Z</t>
+  </si>
+  <si>
+    <t>us/en/adventures/cycling-southern-utah.report.json</t>
+  </si>
+  <si>
+    <t>us/en/adventures/cycling-southern-utah</t>
+  </si>
+  <si>
+    <t>2026-08-12T11:14:01.771Z</t>
+  </si>
+  <si>
+    <t>us/en/adventures/cycling-tuscany.report.json</t>
+  </si>
+  <si>
+    <t>us/en/adventures/cycling-tuscany</t>
+  </si>
+  <si>
+    <t>2026-08-12T11:14:08.370Z</t>
+  </si>
+  <si>
+    <t>us/en/adventures/downhill-skiing-wyoming.report.json</t>
+  </si>
+  <si>
+    <t>us/en/adventures/downhill-skiing-wyoming</t>
+  </si>
+  <si>
+    <t>2026-08-12T11:14:14.332Z</t>
+  </si>
+  <si>
+    <t>us/en/adventures/gastronomic-marais-tour.report.json</t>
+  </si>
+  <si>
+    <t>us/en/adventures/gastronomic-marais-tour</t>
+  </si>
+  <si>
+    <t>2026-08-12T11:14:20.890Z</t>
+  </si>
+  <si>
+    <t>us/en/adventures/napa-wine-tasting.report.json</t>
+  </si>
+  <si>
+    <t>us/en/adventures/napa-wine-tasting</t>
+  </si>
+  <si>
+    <t>2026-08-12T11:14:27.665Z</t>
+  </si>
+  <si>
+    <t>us/en/adventures/riverside-camping-australia.report.json</t>
+  </si>
+  <si>
+    <t>us/en/adventures/riverside-camping-australia</t>
+  </si>
+  <si>
+    <t>2026-08-12T11:14:32.303Z</t>
+  </si>
+  <si>
+    <t>us/en/adventures/ski-touring-mont-blanc.report.json</t>
+  </si>
+  <si>
+    <t>us/en/adventures/ski-touring-mont-blanc</t>
+  </si>
+  <si>
+    <t>2026-08-12T11:14:36.207Z</t>
+  </si>
+  <si>
+    <t>us/en/adventures/surf-camp-costa-rica.report.json</t>
+  </si>
+  <si>
+    <t>us/en/adventures/surf-camp-costa-rica</t>
+  </si>
+  <si>
+    <t>2026-08-12T11:14:40.687Z</t>
+  </si>
+  <si>
+    <t>us/en/adventures/tahoe-skiing.report.json</t>
+  </si>
+  <si>
+    <t>us/en/adventures/tahoe-skiing</t>
+  </si>
+  <si>
+    <t>2026-08-12T11:14:47.245Z</t>
+  </si>
+  <si>
+    <t>us/en/adventures/west-coast-cycling.report.json</t>
+  </si>
+  <si>
+    <t>us/en/adventures/west-coast-cycling</t>
+  </si>
+  <si>
+    <t>2026-08-12T11:14:52.150Z</t>
+  </si>
+  <si>
+    <t>us/en/adventures/whistler-mountain-biking.report.json</t>
+  </si>
+  <si>
+    <t>us/en/adventures/whistler-mountain-biking</t>
+  </si>
+  <si>
+    <t>2026-08-12T11:14:57.767Z</t>
   </si>
   <si>
     <t>us/en/adventures/yosemite-backpacking.html.report.json</t>
@@ -628,6 +781,60 @@
   </si>
   <si>
     <t>2026-08-10T09:12:25.649Z</t>
+  </si>
+  <si>
+    <t>us/en/adventures/yosemite-backpacking.report.json</t>
+  </si>
+  <si>
+    <t>us/en/adventures/yosemite-backpacking</t>
+  </si>
+  <si>
+    <t>2026-08-12T11:15:01.781Z</t>
+  </si>
+  <si>
+    <t>us/en/magazine/arctic-surfing.report.json</t>
+  </si>
+  <si>
+    <t>us/en/magazine/arctic-surfing</t>
+  </si>
+  <si>
+    <t>2026-08-12T11:13:13.925Z</t>
+  </si>
+  <si>
+    <t>us/en/magazine/guide-la-skateparks.report.json</t>
+  </si>
+  <si>
+    <t>us/en/magazine/guide-la-skateparks</t>
+  </si>
+  <si>
+    <t>2026-08-12T11:13:18.992Z</t>
+  </si>
+  <si>
+    <t>us/en/magazine/san-diego-surf.report.json</t>
+  </si>
+  <si>
+    <t>us/en/magazine/san-diego-surf</t>
+  </si>
+  <si>
+    <t>2026-08-12T11:13:25.163Z</t>
+  </si>
+  <si>
+    <t>us/en/magazine/ski-touring.report.json</t>
+  </si>
+  <si>
+    <t>us/en/magazine/ski-touring</t>
+  </si>
+  <si>
+    <t>2026-08-12T11:13:30.153Z</t>
+  </si>
+  <si>
+    <t>us/en/magazine/western-australia.report.json</t>
+  </si>
+  <si>
+    <t>us/en/magazine/western-australia</t>
+  </si>
+  <si>
+    <t>2026-08-12T11:13:35.310Z</t>
   </si>
 </sst>
 </file>
@@ -1016,11 +1223,11 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:J39"/>
+  <dimension ref="A1:J62"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="4" width="50" customWidth="1"/>
-    <col min="5" max="5" width="44" customWidth="1"/>
+    <col min="5" max="5" width="46" customWidth="1"/>
     <col min="7" max="7" width="17" customWidth="1"/>
     <col min="8" max="8" width="26" customWidth="1"/>
     <col min="9" max="10" width="50" customWidth="1"/>
@@ -2183,7 +2390,7 @@
         <v>193</v>
       </c>
       <c r="B37" t="s">
-        <v>41</v>
+        <v>20</v>
       </c>
       <c r="C37" t="s">
         <v>12</v>
@@ -2198,16 +2405,16 @@
         <v>14</v>
       </c>
       <c r="G37" t="s">
-        <v>43</v>
+        <v>22</v>
       </c>
       <c r="H37" t="s">
         <v>195</v>
       </c>
       <c r="I37" t="s">
-        <v>45</v>
+        <v>24</v>
       </c>
       <c r="J37" t="s">
-        <v>46</v>
+        <v>25</v>
       </c>
     </row>
     <row r="38" spans="1:10" x14ac:dyDescent="0.25">
@@ -2215,7 +2422,7 @@
         <v>196</v>
       </c>
       <c r="B38" t="s">
-        <v>34</v>
+        <v>41</v>
       </c>
       <c r="C38" t="s">
         <v>12</v>
@@ -2230,16 +2437,16 @@
         <v>14</v>
       </c>
       <c r="G38" t="s">
-        <v>36</v>
+        <v>43</v>
       </c>
       <c r="H38" t="s">
         <v>198</v>
       </c>
       <c r="I38" t="s">
-        <v>38</v>
+        <v>45</v>
       </c>
       <c r="J38" t="s">
-        <v>39</v>
+        <v>46</v>
       </c>
     </row>
     <row r="39" spans="1:10" x14ac:dyDescent="0.25">
@@ -2247,31 +2454,767 @@
         <v>199</v>
       </c>
       <c r="B39" t="s">
-        <v>12</v>
+        <v>34</v>
       </c>
       <c r="C39" t="s">
+        <v>12</v>
+      </c>
+      <c r="D39" t="s">
+        <v>12</v>
+      </c>
+      <c r="E39" t="s">
         <v>200</v>
       </c>
-      <c r="D39" t="s">
+      <c r="F39" t="s">
+        <v>14</v>
+      </c>
+      <c r="G39" t="s">
+        <v>36</v>
+      </c>
+      <c r="H39" t="s">
         <v>201</v>
       </c>
-      <c r="E39" t="s">
+      <c r="I39" t="s">
+        <v>38</v>
+      </c>
+      <c r="J39" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="40" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A40" t="s">
         <v>202</v>
       </c>
-      <c r="F39" t="s">
+      <c r="B40" t="s">
+        <v>12</v>
+      </c>
+      <c r="C40" t="s">
+        <v>12</v>
+      </c>
+      <c r="D40" t="s">
+        <v>12</v>
+      </c>
+      <c r="E40" t="s">
         <v>203</v>
       </c>
-      <c r="G39" t="s">
-        <v>12</v>
-      </c>
-      <c r="H39" t="s">
+      <c r="F40" t="s">
+        <v>14</v>
+      </c>
+      <c r="G40" t="s">
+        <v>69</v>
+      </c>
+      <c r="H40" t="s">
         <v>204</v>
       </c>
-      <c r="I39" t="s">
-        <v>12</v>
-      </c>
-      <c r="J39" t="s">
+      <c r="I40" t="s">
+        <v>71</v>
+      </c>
+      <c r="J40" t="s">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="41" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A41" t="s">
+        <v>205</v>
+      </c>
+      <c r="B41" t="s">
+        <v>73</v>
+      </c>
+      <c r="C41" t="s">
+        <v>12</v>
+      </c>
+      <c r="D41" t="s">
+        <v>12</v>
+      </c>
+      <c r="E41" t="s">
+        <v>206</v>
+      </c>
+      <c r="F41" t="s">
+        <v>14</v>
+      </c>
+      <c r="G41" t="s">
+        <v>75</v>
+      </c>
+      <c r="H41" t="s">
+        <v>207</v>
+      </c>
+      <c r="I41" t="s">
+        <v>77</v>
+      </c>
+      <c r="J41" t="s">
+        <v>78</v>
+      </c>
+    </row>
+    <row r="42" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A42" t="s">
+        <v>208</v>
+      </c>
+      <c r="B42" t="s">
+        <v>73</v>
+      </c>
+      <c r="C42" t="s">
+        <v>12</v>
+      </c>
+      <c r="D42" t="s">
+        <v>12</v>
+      </c>
+      <c r="E42" t="s">
+        <v>209</v>
+      </c>
+      <c r="F42" t="s">
+        <v>14</v>
+      </c>
+      <c r="G42" t="s">
+        <v>75</v>
+      </c>
+      <c r="H42" t="s">
+        <v>210</v>
+      </c>
+      <c r="I42" t="s">
+        <v>82</v>
+      </c>
+      <c r="J42" t="s">
+        <v>83</v>
+      </c>
+    </row>
+    <row r="43" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A43" t="s">
+        <v>211</v>
+      </c>
+      <c r="B43" t="s">
+        <v>73</v>
+      </c>
+      <c r="C43" t="s">
+        <v>12</v>
+      </c>
+      <c r="D43" t="s">
+        <v>12</v>
+      </c>
+      <c r="E43" t="s">
+        <v>212</v>
+      </c>
+      <c r="F43" t="s">
+        <v>14</v>
+      </c>
+      <c r="G43" t="s">
+        <v>75</v>
+      </c>
+      <c r="H43" t="s">
+        <v>213</v>
+      </c>
+      <c r="I43" t="s">
+        <v>87</v>
+      </c>
+      <c r="J43" t="s">
+        <v>88</v>
+      </c>
+    </row>
+    <row r="44" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A44" t="s">
+        <v>214</v>
+      </c>
+      <c r="B44" t="s">
+        <v>73</v>
+      </c>
+      <c r="C44" t="s">
+        <v>12</v>
+      </c>
+      <c r="D44" t="s">
+        <v>12</v>
+      </c>
+      <c r="E44" t="s">
+        <v>215</v>
+      </c>
+      <c r="F44" t="s">
+        <v>14</v>
+      </c>
+      <c r="G44" t="s">
+        <v>75</v>
+      </c>
+      <c r="H44" t="s">
+        <v>216</v>
+      </c>
+      <c r="I44" t="s">
+        <v>92</v>
+      </c>
+      <c r="J44" t="s">
+        <v>93</v>
+      </c>
+    </row>
+    <row r="45" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A45" t="s">
+        <v>217</v>
+      </c>
+      <c r="B45" t="s">
+        <v>73</v>
+      </c>
+      <c r="C45" t="s">
+        <v>12</v>
+      </c>
+      <c r="D45" t="s">
+        <v>12</v>
+      </c>
+      <c r="E45" t="s">
+        <v>218</v>
+      </c>
+      <c r="F45" t="s">
+        <v>14</v>
+      </c>
+      <c r="G45" t="s">
+        <v>75</v>
+      </c>
+      <c r="H45" t="s">
+        <v>219</v>
+      </c>
+      <c r="I45" t="s">
+        <v>97</v>
+      </c>
+      <c r="J45" t="s">
+        <v>98</v>
+      </c>
+    </row>
+    <row r="46" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A46" t="s">
+        <v>220</v>
+      </c>
+      <c r="B46" t="s">
+        <v>73</v>
+      </c>
+      <c r="C46" t="s">
+        <v>12</v>
+      </c>
+      <c r="D46" t="s">
+        <v>12</v>
+      </c>
+      <c r="E46" t="s">
+        <v>221</v>
+      </c>
+      <c r="F46" t="s">
+        <v>14</v>
+      </c>
+      <c r="G46" t="s">
+        <v>75</v>
+      </c>
+      <c r="H46" t="s">
+        <v>222</v>
+      </c>
+      <c r="I46" t="s">
+        <v>102</v>
+      </c>
+      <c r="J46" t="s">
+        <v>103</v>
+      </c>
+    </row>
+    <row r="47" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A47" t="s">
+        <v>223</v>
+      </c>
+      <c r="B47" t="s">
+        <v>73</v>
+      </c>
+      <c r="C47" t="s">
+        <v>12</v>
+      </c>
+      <c r="D47" t="s">
+        <v>12</v>
+      </c>
+      <c r="E47" t="s">
+        <v>224</v>
+      </c>
+      <c r="F47" t="s">
+        <v>14</v>
+      </c>
+      <c r="G47" t="s">
+        <v>75</v>
+      </c>
+      <c r="H47" t="s">
+        <v>225</v>
+      </c>
+      <c r="I47" t="s">
+        <v>107</v>
+      </c>
+      <c r="J47" t="s">
+        <v>108</v>
+      </c>
+    </row>
+    <row r="48" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A48" t="s">
+        <v>226</v>
+      </c>
+      <c r="B48" t="s">
+        <v>73</v>
+      </c>
+      <c r="C48" t="s">
+        <v>12</v>
+      </c>
+      <c r="D48" t="s">
+        <v>12</v>
+      </c>
+      <c r="E48" t="s">
+        <v>227</v>
+      </c>
+      <c r="F48" t="s">
+        <v>14</v>
+      </c>
+      <c r="G48" t="s">
+        <v>75</v>
+      </c>
+      <c r="H48" t="s">
+        <v>228</v>
+      </c>
+      <c r="I48" t="s">
+        <v>112</v>
+      </c>
+      <c r="J48" t="s">
+        <v>113</v>
+      </c>
+    </row>
+    <row r="49" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A49" t="s">
+        <v>229</v>
+      </c>
+      <c r="B49" t="s">
+        <v>73</v>
+      </c>
+      <c r="C49" t="s">
+        <v>12</v>
+      </c>
+      <c r="D49" t="s">
+        <v>12</v>
+      </c>
+      <c r="E49" t="s">
+        <v>230</v>
+      </c>
+      <c r="F49" t="s">
+        <v>14</v>
+      </c>
+      <c r="G49" t="s">
+        <v>75</v>
+      </c>
+      <c r="H49" t="s">
+        <v>231</v>
+      </c>
+      <c r="I49" t="s">
+        <v>117</v>
+      </c>
+      <c r="J49" t="s">
+        <v>118</v>
+      </c>
+    </row>
+    <row r="50" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A50" t="s">
+        <v>232</v>
+      </c>
+      <c r="B50" t="s">
+        <v>73</v>
+      </c>
+      <c r="C50" t="s">
+        <v>12</v>
+      </c>
+      <c r="D50" t="s">
+        <v>12</v>
+      </c>
+      <c r="E50" t="s">
+        <v>233</v>
+      </c>
+      <c r="F50" t="s">
+        <v>14</v>
+      </c>
+      <c r="G50" t="s">
+        <v>75</v>
+      </c>
+      <c r="H50" t="s">
+        <v>234</v>
+      </c>
+      <c r="I50" t="s">
+        <v>122</v>
+      </c>
+      <c r="J50" t="s">
+        <v>123</v>
+      </c>
+    </row>
+    <row r="51" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A51" t="s">
+        <v>235</v>
+      </c>
+      <c r="B51" t="s">
+        <v>73</v>
+      </c>
+      <c r="C51" t="s">
+        <v>12</v>
+      </c>
+      <c r="D51" t="s">
+        <v>12</v>
+      </c>
+      <c r="E51" t="s">
+        <v>236</v>
+      </c>
+      <c r="F51" t="s">
+        <v>14</v>
+      </c>
+      <c r="G51" t="s">
+        <v>75</v>
+      </c>
+      <c r="H51" t="s">
+        <v>237</v>
+      </c>
+      <c r="I51" t="s">
+        <v>127</v>
+      </c>
+      <c r="J51" t="s">
+        <v>128</v>
+      </c>
+    </row>
+    <row r="52" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A52" t="s">
+        <v>238</v>
+      </c>
+      <c r="B52" t="s">
+        <v>73</v>
+      </c>
+      <c r="C52" t="s">
+        <v>12</v>
+      </c>
+      <c r="D52" t="s">
+        <v>12</v>
+      </c>
+      <c r="E52" t="s">
+        <v>239</v>
+      </c>
+      <c r="F52" t="s">
+        <v>14</v>
+      </c>
+      <c r="G52" t="s">
+        <v>75</v>
+      </c>
+      <c r="H52" t="s">
+        <v>240</v>
+      </c>
+      <c r="I52" t="s">
+        <v>132</v>
+      </c>
+      <c r="J52" t="s">
+        <v>133</v>
+      </c>
+    </row>
+    <row r="53" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A53" t="s">
+        <v>241</v>
+      </c>
+      <c r="B53" t="s">
+        <v>73</v>
+      </c>
+      <c r="C53" t="s">
+        <v>12</v>
+      </c>
+      <c r="D53" t="s">
+        <v>12</v>
+      </c>
+      <c r="E53" t="s">
+        <v>242</v>
+      </c>
+      <c r="F53" t="s">
+        <v>14</v>
+      </c>
+      <c r="G53" t="s">
+        <v>75</v>
+      </c>
+      <c r="H53" t="s">
+        <v>243</v>
+      </c>
+      <c r="I53" t="s">
+        <v>137</v>
+      </c>
+      <c r="J53" t="s">
+        <v>138</v>
+      </c>
+    </row>
+    <row r="54" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A54" t="s">
+        <v>244</v>
+      </c>
+      <c r="B54" t="s">
+        <v>73</v>
+      </c>
+      <c r="C54" t="s">
+        <v>12</v>
+      </c>
+      <c r="D54" t="s">
+        <v>12</v>
+      </c>
+      <c r="E54" t="s">
+        <v>245</v>
+      </c>
+      <c r="F54" t="s">
+        <v>14</v>
+      </c>
+      <c r="G54" t="s">
+        <v>75</v>
+      </c>
+      <c r="H54" t="s">
+        <v>246</v>
+      </c>
+      <c r="I54" t="s">
+        <v>142</v>
+      </c>
+      <c r="J54" t="s">
+        <v>143</v>
+      </c>
+    </row>
+    <row r="55" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A55" t="s">
+        <v>247</v>
+      </c>
+      <c r="B55" t="s">
+        <v>73</v>
+      </c>
+      <c r="C55" t="s">
+        <v>12</v>
+      </c>
+      <c r="D55" t="s">
+        <v>12</v>
+      </c>
+      <c r="E55" t="s">
+        <v>248</v>
+      </c>
+      <c r="F55" t="s">
+        <v>14</v>
+      </c>
+      <c r="G55" t="s">
+        <v>75</v>
+      </c>
+      <c r="H55" t="s">
+        <v>249</v>
+      </c>
+      <c r="I55" t="s">
+        <v>147</v>
+      </c>
+      <c r="J55" t="s">
+        <v>148</v>
+      </c>
+    </row>
+    <row r="56" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A56" t="s">
+        <v>250</v>
+      </c>
+      <c r="B56" t="s">
+        <v>12</v>
+      </c>
+      <c r="C56" t="s">
+        <v>251</v>
+      </c>
+      <c r="D56" t="s">
+        <v>252</v>
+      </c>
+      <c r="E56" t="s">
+        <v>253</v>
+      </c>
+      <c r="F56" t="s">
+        <v>254</v>
+      </c>
+      <c r="G56" t="s">
+        <v>12</v>
+      </c>
+      <c r="H56" t="s">
+        <v>255</v>
+      </c>
+      <c r="I56" t="s">
+        <v>12</v>
+      </c>
+      <c r="J56" t="s">
         <v>153</v>
+      </c>
+    </row>
+    <row r="57" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A57" t="s">
+        <v>256</v>
+      </c>
+      <c r="B57" t="s">
+        <v>73</v>
+      </c>
+      <c r="C57" t="s">
+        <v>12</v>
+      </c>
+      <c r="D57" t="s">
+        <v>12</v>
+      </c>
+      <c r="E57" t="s">
+        <v>257</v>
+      </c>
+      <c r="F57" t="s">
+        <v>14</v>
+      </c>
+      <c r="G57" t="s">
+        <v>75</v>
+      </c>
+      <c r="H57" t="s">
+        <v>258</v>
+      </c>
+      <c r="I57" t="s">
+        <v>152</v>
+      </c>
+      <c r="J57" t="s">
+        <v>153</v>
+      </c>
+    </row>
+    <row r="58" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A58" t="s">
+        <v>259</v>
+      </c>
+      <c r="B58" t="s">
+        <v>27</v>
+      </c>
+      <c r="C58" t="s">
+        <v>12</v>
+      </c>
+      <c r="D58" t="s">
+        <v>12</v>
+      </c>
+      <c r="E58" t="s">
+        <v>260</v>
+      </c>
+      <c r="F58" t="s">
+        <v>14</v>
+      </c>
+      <c r="G58" t="s">
+        <v>29</v>
+      </c>
+      <c r="H58" t="s">
+        <v>261</v>
+      </c>
+      <c r="I58" t="s">
+        <v>31</v>
+      </c>
+      <c r="J58" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="59" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A59" t="s">
+        <v>262</v>
+      </c>
+      <c r="B59" t="s">
+        <v>27</v>
+      </c>
+      <c r="C59" t="s">
+        <v>12</v>
+      </c>
+      <c r="D59" t="s">
+        <v>12</v>
+      </c>
+      <c r="E59" t="s">
+        <v>263</v>
+      </c>
+      <c r="F59" t="s">
+        <v>14</v>
+      </c>
+      <c r="G59" t="s">
+        <v>29</v>
+      </c>
+      <c r="H59" t="s">
+        <v>264</v>
+      </c>
+      <c r="I59" t="s">
+        <v>170</v>
+      </c>
+      <c r="J59" t="s">
+        <v>171</v>
+      </c>
+    </row>
+    <row r="60" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A60" t="s">
+        <v>265</v>
+      </c>
+      <c r="B60" t="s">
+        <v>27</v>
+      </c>
+      <c r="C60" t="s">
+        <v>12</v>
+      </c>
+      <c r="D60" t="s">
+        <v>12</v>
+      </c>
+      <c r="E60" t="s">
+        <v>266</v>
+      </c>
+      <c r="F60" t="s">
+        <v>14</v>
+      </c>
+      <c r="G60" t="s">
+        <v>29</v>
+      </c>
+      <c r="H60" t="s">
+        <v>267</v>
+      </c>
+      <c r="I60" t="s">
+        <v>175</v>
+      </c>
+      <c r="J60" t="s">
+        <v>176</v>
+      </c>
+    </row>
+    <row r="61" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A61" t="s">
+        <v>268</v>
+      </c>
+      <c r="B61" t="s">
+        <v>27</v>
+      </c>
+      <c r="C61" t="s">
+        <v>12</v>
+      </c>
+      <c r="D61" t="s">
+        <v>12</v>
+      </c>
+      <c r="E61" t="s">
+        <v>269</v>
+      </c>
+      <c r="F61" t="s">
+        <v>14</v>
+      </c>
+      <c r="G61" t="s">
+        <v>29</v>
+      </c>
+      <c r="H61" t="s">
+        <v>270</v>
+      </c>
+      <c r="I61" t="s">
+        <v>180</v>
+      </c>
+      <c r="J61" t="s">
+        <v>181</v>
+      </c>
+    </row>
+    <row r="62" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A62" t="s">
+        <v>271</v>
+      </c>
+      <c r="B62" t="s">
+        <v>27</v>
+      </c>
+      <c r="C62" t="s">
+        <v>12</v>
+      </c>
+      <c r="D62" t="s">
+        <v>12</v>
+      </c>
+      <c r="E62" t="s">
+        <v>272</v>
+      </c>
+      <c r="F62" t="s">
+        <v>14</v>
+      </c>
+      <c r="G62" t="s">
+        <v>29</v>
+      </c>
+      <c r="H62" t="s">
+        <v>273</v>
+      </c>
+      <c r="I62" t="s">
+        <v>185</v>
+      </c>
+      <c r="J62" t="s">
+        <v>186</v>
       </c>
     </row>
   </sheetData>

</xml_diff>